<commit_message>
update Waarnemingen and Add Heikikker, GladdeSlang en Modderkruiper
</commit_message>
<xml_diff>
--- a/data/input/Excel_files/Soorten_bwk_afstanden.xlsx
+++ b/data/input/Excel_files/Soorten_bwk_afstanden.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bert_vanhecke\Documents\Soortenbehoud\Turnhouts Vennegebied\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bert_vanhecke\Documents\Soortenbehoud\arpl\data\input\Excel_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -1281,7 +1281,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:L322"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1329,7 +1328,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -1358,7 +1357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -1384,7 +1383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -1410,7 +1409,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -1436,7 +1435,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -1462,7 +1461,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -1488,7 +1487,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -1514,7 +1513,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -1540,7 +1539,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -1566,7 +1565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>18</v>
       </c>
@@ -1592,7 +1591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>16</v>
       </c>
@@ -1621,7 +1620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>18</v>
       </c>
@@ -1647,7 +1646,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -1673,7 +1672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -1696,7 +1695,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>18</v>
       </c>
@@ -1722,7 +1721,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>18</v>
       </c>
@@ -1748,7 +1747,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>21</v>
       </c>
@@ -1777,7 +1776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>21</v>
       </c>
@@ -1806,7 +1805,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>21</v>
       </c>
@@ -1826,7 +1825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -1852,7 +1851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>44</v>
       </c>
@@ -1881,7 +1880,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -1907,7 +1906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>21</v>
       </c>
@@ -1933,7 +1932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>21</v>
       </c>
@@ -2915,7 +2914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>16</v>
       </c>
@@ -3335,7 +3334,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>44</v>
       </c>
@@ -3364,7 +3363,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>44</v>
       </c>
@@ -3393,7 +3392,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>44</v>
       </c>
@@ -3422,7 +3421,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>44</v>
       </c>
@@ -3451,7 +3450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>44</v>
       </c>
@@ -3480,7 +3479,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>44</v>
       </c>
@@ -3509,7 +3508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>190</v>
       </c>
@@ -3535,7 +3534,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>44</v>
       </c>
@@ -3564,7 +3563,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>16</v>
       </c>
@@ -3593,7 +3592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>44</v>
       </c>
@@ -3622,7 +3621,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>16</v>
       </c>
@@ -3648,7 +3647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>44</v>
       </c>
@@ -3677,7 +3676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>44</v>
       </c>
@@ -3706,7 +3705,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="88" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>44</v>
       </c>
@@ -3735,7 +3734,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>44</v>
       </c>
@@ -3764,7 +3763,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>44</v>
       </c>
@@ -3793,7 +3792,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>44</v>
       </c>
@@ -3822,7 +3821,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>44</v>
       </c>
@@ -3851,7 +3850,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>44</v>
       </c>
@@ -3880,7 +3879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>16</v>
       </c>
@@ -3909,7 +3908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>44</v>
       </c>
@@ -3939,7 +3938,7 @@
       </c>
       <c r="L95" s="1"/>
     </row>
-    <row r="96" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>44</v>
       </c>
@@ -3968,7 +3967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>191</v>
       </c>
@@ -3997,7 +3996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>44</v>
       </c>
@@ -4026,7 +4025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>190</v>
       </c>
@@ -4081,7 +4080,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>32</v>
       </c>
@@ -4107,7 +4106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>16</v>
       </c>
@@ -4136,7 +4135,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>44</v>
       </c>
@@ -4165,7 +4164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>44</v>
       </c>
@@ -4194,7 +4193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>44</v>
       </c>
@@ -4223,7 +4222,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>190</v>
       </c>
@@ -4252,7 +4251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>44</v>
       </c>
@@ -4281,7 +4280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>16</v>
       </c>
@@ -4310,7 +4309,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>44</v>
       </c>
@@ -4339,7 +4338,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>44</v>
       </c>
@@ -4368,7 +4367,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>44</v>
       </c>
@@ -4397,7 +4396,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>44</v>
       </c>
@@ -4426,7 +4425,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>18</v>
       </c>
@@ -4452,7 +4451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>16</v>
       </c>
@@ -4481,7 +4480,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>44</v>
       </c>
@@ -4510,7 +4509,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>44</v>
       </c>
@@ -4539,7 +4538,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>44</v>
       </c>
@@ -4568,7 +4567,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>190</v>
       </c>
@@ -4594,7 +4593,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>44</v>
       </c>
@@ -4623,7 +4622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>16</v>
       </c>
@@ -4649,7 +4648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>16</v>
       </c>
@@ -4678,7 +4677,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>44</v>
       </c>
@@ -4707,7 +4706,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>16</v>
       </c>
@@ -4736,7 +4735,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>44</v>
       </c>
@@ -4765,7 +4764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>16</v>
       </c>
@@ -4794,7 +4793,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>16</v>
       </c>
@@ -4823,7 +4822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>44</v>
       </c>
@@ -4852,7 +4851,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>44</v>
       </c>
@@ -4881,7 +4880,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>44</v>
       </c>
@@ -4910,7 +4909,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>44</v>
       </c>
@@ -4939,7 +4938,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>44</v>
       </c>
@@ -4968,7 +4967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>44</v>
       </c>
@@ -4997,7 +4996,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>44</v>
       </c>
@@ -5026,7 +5025,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>44</v>
       </c>
@@ -5055,7 +5054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>190</v>
       </c>
@@ -5081,7 +5080,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>190</v>
       </c>
@@ -5107,7 +5106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>44</v>
       </c>
@@ -5136,7 +5135,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>44</v>
       </c>
@@ -5165,7 +5164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>190</v>
       </c>
@@ -5194,7 +5193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>44</v>
       </c>
@@ -5223,7 +5222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>44</v>
       </c>
@@ -5252,7 +5251,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>44</v>
       </c>
@@ -5281,7 +5280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>40</v>
       </c>
@@ -5310,7 +5309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>18</v>
       </c>
@@ -5336,7 +5335,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>44</v>
       </c>
@@ -5365,7 +5364,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>44</v>
       </c>
@@ -5394,7 +5393,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>44</v>
       </c>
@@ -5423,7 +5422,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>44</v>
       </c>
@@ -5452,7 +5451,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>190</v>
       </c>
@@ -5478,7 +5477,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>16</v>
       </c>
@@ -5504,7 +5503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>44</v>
       </c>
@@ -5533,7 +5532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>190</v>
       </c>
@@ -5562,7 +5561,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>44</v>
       </c>
@@ -5591,7 +5590,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>190</v>
       </c>
@@ -5617,7 +5616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>44</v>
       </c>
@@ -5646,7 +5645,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>44</v>
       </c>
@@ -5675,7 +5674,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>44</v>
       </c>
@@ -5704,7 +5703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>44</v>
       </c>
@@ -5733,7 +5732,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>43</v>
       </c>
@@ -5759,7 +5758,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>43</v>
       </c>
@@ -5785,7 +5784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>43</v>
       </c>
@@ -5811,7 +5810,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>43</v>
       </c>
@@ -5837,7 +5836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>40</v>
       </c>
@@ -5866,7 +5865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>44</v>
       </c>
@@ -5895,7 +5894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>223</v>
       </c>
@@ -5924,7 +5923,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="166" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>223</v>
       </c>
@@ -5953,7 +5952,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>223</v>
       </c>
@@ -5982,7 +5981,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>223</v>
       </c>
@@ -6011,7 +6010,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>223</v>
       </c>
@@ -6040,7 +6039,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>223</v>
       </c>
@@ -6069,7 +6068,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>223</v>
       </c>
@@ -6098,7 +6097,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>223</v>
       </c>
@@ -6127,7 +6126,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>223</v>
       </c>
@@ -6156,7 +6155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>41</v>
       </c>
@@ -6172,6 +6171,9 @@
       <c r="E174">
         <v>10</v>
       </c>
+      <c r="F174">
+        <v>1500</v>
+      </c>
       <c r="G174" t="s">
         <v>274</v>
       </c>
@@ -6182,7 +6184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>16</v>
       </c>
@@ -6208,7 +6210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>16</v>
       </c>
@@ -6237,7 +6239,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="177" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>16</v>
       </c>
@@ -6266,7 +6268,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="178" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>16</v>
       </c>
@@ -6295,7 +6297,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="179" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>16</v>
       </c>
@@ -6324,7 +6326,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="180" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>190</v>
       </c>
@@ -6350,7 +6352,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>44</v>
       </c>
@@ -6379,7 +6381,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="182" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>44</v>
       </c>
@@ -6408,7 +6410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="183" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>16</v>
       </c>
@@ -6437,7 +6439,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="184" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>16</v>
       </c>
@@ -6466,7 +6468,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="185" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>16</v>
       </c>
@@ -6495,7 +6497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>16</v>
       </c>
@@ -6524,7 +6526,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>44</v>
       </c>
@@ -6553,7 +6555,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>44</v>
       </c>
@@ -6582,7 +6584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>44</v>
       </c>
@@ -6611,7 +6613,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>16</v>
       </c>
@@ -6640,7 +6642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>44</v>
       </c>
@@ -6669,7 +6671,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>44</v>
       </c>
@@ -6698,7 +6700,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="193" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>44</v>
       </c>
@@ -6727,7 +6729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>190</v>
       </c>
@@ -6756,7 +6758,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>16</v>
       </c>
@@ -6785,7 +6787,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="196" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>16</v>
       </c>
@@ -6814,7 +6816,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="197" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>16</v>
       </c>
@@ -6840,7 +6842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>44</v>
       </c>
@@ -6869,7 +6871,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="199" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>44</v>
       </c>
@@ -6898,7 +6900,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="200" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>16</v>
       </c>
@@ -6924,7 +6926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>16</v>
       </c>
@@ -6950,7 +6952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>44</v>
       </c>
@@ -6979,7 +6981,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="203" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>44</v>
       </c>
@@ -7008,7 +7010,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="204" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>44</v>
       </c>
@@ -7037,7 +7039,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>44</v>
       </c>
@@ -7066,7 +7068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>190</v>
       </c>
@@ -7095,7 +7097,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="207" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>190</v>
       </c>
@@ -7124,7 +7126,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>190</v>
       </c>
@@ -7153,7 +7155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>190</v>
       </c>
@@ -7182,7 +7184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="210" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>44</v>
       </c>
@@ -7211,7 +7213,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="211" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>190</v>
       </c>
@@ -7240,7 +7242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>190</v>
       </c>
@@ -7269,7 +7271,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="213" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>190</v>
       </c>
@@ -7298,7 +7300,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="214" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>44</v>
       </c>
@@ -7327,7 +7329,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="215" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>190</v>
       </c>
@@ -7353,7 +7355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>190</v>
       </c>
@@ -7382,7 +7384,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>190</v>
       </c>
@@ -7408,7 +7410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="218" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>190</v>
       </c>
@@ -7434,7 +7436,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="219" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>190</v>
       </c>
@@ -7460,7 +7462,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="220" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>44</v>
       </c>
@@ -7490,7 +7492,7 @@
       </c>
       <c r="L220" s="1"/>
     </row>
-    <row r="221" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>190</v>
       </c>
@@ -7516,7 +7518,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="222" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>190</v>
       </c>
@@ -7542,7 +7544,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="223" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>190</v>
       </c>
@@ -7568,7 +7570,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>190</v>
       </c>
@@ -7594,7 +7596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>190</v>
       </c>
@@ -7620,7 +7622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>44</v>
       </c>
@@ -7649,7 +7651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>190</v>
       </c>
@@ -7675,7 +7677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>190</v>
       </c>
@@ -7701,7 +7703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>190</v>
       </c>
@@ -7727,7 +7729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>190</v>
       </c>
@@ -7753,7 +7755,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="231" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>190</v>
       </c>
@@ -7779,7 +7781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="232" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>190</v>
       </c>
@@ -7805,7 +7807,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="233" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>190</v>
       </c>
@@ -7831,7 +7833,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="234" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>190</v>
       </c>
@@ -7857,7 +7859,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="235" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>190</v>
       </c>
@@ -7883,7 +7885,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="236" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>190</v>
       </c>
@@ -7909,7 +7911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="237" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>190</v>
       </c>
@@ -7935,7 +7937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="238" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>190</v>
       </c>
@@ -7961,7 +7963,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="239" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>190</v>
       </c>
@@ -7987,7 +7989,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="240" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>190</v>
       </c>
@@ -8013,7 +8015,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="241" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>44</v>
       </c>
@@ -8042,7 +8044,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="242" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>190</v>
       </c>
@@ -8068,7 +8070,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="243" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>190</v>
       </c>
@@ -8094,7 +8096,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="244" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>190</v>
       </c>
@@ -8120,7 +8122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="245" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>190</v>
       </c>
@@ -8146,7 +8148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="246" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>190</v>
       </c>
@@ -8172,7 +8174,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="247" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>190</v>
       </c>
@@ -8198,7 +8200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>190</v>
       </c>
@@ -8224,7 +8226,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="249" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>190</v>
       </c>
@@ -8250,7 +8252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="250" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>190</v>
       </c>
@@ -8276,7 +8278,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="251" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>44</v>
       </c>
@@ -8305,7 +8307,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="252" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>190</v>
       </c>
@@ -8331,7 +8333,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="253" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>190</v>
       </c>
@@ -8357,7 +8359,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="254" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>190</v>
       </c>
@@ -8383,7 +8385,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="255" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>190</v>
       </c>
@@ -8409,7 +8411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="256" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>190</v>
       </c>
@@ -8435,7 +8437,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>190</v>
       </c>
@@ -8461,7 +8463,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="258" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
         <v>190</v>
       </c>
@@ -8487,7 +8489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="259" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>190</v>
       </c>
@@ -8513,7 +8515,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>44</v>
       </c>
@@ -8542,7 +8544,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="261" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>190</v>
       </c>
@@ -8568,7 +8570,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="262" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>190</v>
       </c>
@@ -8594,7 +8596,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="263" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>190</v>
       </c>
@@ -8620,7 +8622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="264" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>44</v>
       </c>
@@ -8649,7 +8651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="265" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>190</v>
       </c>
@@ -8675,7 +8677,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="266" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>190</v>
       </c>
@@ -8701,7 +8703,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="267" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>190</v>
       </c>
@@ -8727,7 +8729,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="268" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>190</v>
       </c>
@@ -8753,7 +8755,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="269" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>190</v>
       </c>
@@ -8779,7 +8781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="270" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
         <v>44</v>
       </c>
@@ -8808,7 +8810,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="271" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>190</v>
       </c>
@@ -8834,7 +8836,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="272" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
         <v>190</v>
       </c>
@@ -8860,7 +8862,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="273" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>190</v>
       </c>
@@ -8886,7 +8888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="274" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>190</v>
       </c>
@@ -8912,7 +8914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="275" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>190</v>
       </c>
@@ -8938,7 +8940,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="276" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
         <v>190</v>
       </c>
@@ -8964,7 +8966,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="277" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
         <v>190</v>
       </c>
@@ -8990,7 +8992,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="278" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
         <v>190</v>
       </c>
@@ -9016,7 +9018,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="279" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>190</v>
       </c>
@@ -9042,7 +9044,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="280" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>190</v>
       </c>
@@ -9068,7 +9070,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="281" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>190</v>
       </c>
@@ -9094,7 +9096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="282" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>190</v>
       </c>
@@ -9120,7 +9122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="283" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>190</v>
       </c>
@@ -9146,7 +9148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="284" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
         <v>190</v>
       </c>
@@ -9172,7 +9174,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="285" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>190</v>
       </c>
@@ -9198,7 +9200,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="286" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>190</v>
       </c>
@@ -9224,7 +9226,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="287" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>190</v>
       </c>
@@ -9250,7 +9252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="288" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>190</v>
       </c>
@@ -9276,7 +9278,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="289" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>190</v>
       </c>
@@ -9302,7 +9304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="290" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
         <v>190</v>
       </c>
@@ -9328,7 +9330,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="291" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>190</v>
       </c>
@@ -9354,7 +9356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="292" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
         <v>44</v>
       </c>
@@ -9383,7 +9385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="293" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
         <v>190</v>
       </c>
@@ -9409,7 +9411,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="294" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
         <v>190</v>
       </c>
@@ -9435,7 +9437,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="295" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
         <v>190</v>
       </c>
@@ -9461,7 +9463,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="296" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>190</v>
       </c>
@@ -9487,7 +9489,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="297" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
         <v>44</v>
       </c>
@@ -9516,7 +9518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="298" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>190</v>
       </c>
@@ -9542,7 +9544,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="299" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>190</v>
       </c>
@@ -9568,7 +9570,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="300" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="300" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
         <v>190</v>
       </c>
@@ -9594,7 +9596,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="301" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>190</v>
       </c>
@@ -9620,7 +9622,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="302" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>190</v>
       </c>
@@ -9646,7 +9648,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="303" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>190</v>
       </c>
@@ -9672,7 +9674,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="304" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>190</v>
       </c>
@@ -9698,7 +9700,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="305" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>190</v>
       </c>
@@ -9724,7 +9726,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="306" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>190</v>
       </c>
@@ -9750,7 +9752,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="307" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>42</v>
       </c>
@@ -9776,7 +9778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="308" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>191</v>
       </c>
@@ -9805,7 +9807,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="309" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
         <v>191</v>
       </c>
@@ -9834,7 +9836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="310" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
         <v>191</v>
       </c>
@@ -9863,7 +9865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="311" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
         <v>191</v>
       </c>
@@ -9892,7 +9894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="312" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
         <v>16</v>
       </c>
@@ -9918,7 +9920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="313" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
         <v>191</v>
       </c>
@@ -9947,7 +9949,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="314" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
         <v>191</v>
       </c>
@@ -9973,7 +9975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="315" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
         <v>191</v>
       </c>
@@ -9999,7 +10001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="316" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
         <v>191</v>
       </c>
@@ -10025,7 +10027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="317" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
         <v>191</v>
       </c>
@@ -10051,7 +10053,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="318" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
         <v>191</v>
       </c>
@@ -10077,7 +10079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="319" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A319" t="s">
         <v>191</v>
       </c>
@@ -10103,7 +10105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="320" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A320" t="s">
         <v>191</v>
       </c>
@@ -10129,7 +10131,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="321" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A321" t="s">
         <v>191</v>
       </c>
@@ -10155,7 +10157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="322" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A322" t="s">
         <v>191</v>
       </c>
@@ -10183,11 +10185,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:I322">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Libellen"/>
-      </filters>
-    </filterColumn>
     <sortState ref="A26:I100">
       <sortCondition ref="B1:B322"/>
     </sortState>

</xml_diff>

<commit_message>
Add Hoogveenglanslibel en Heivlinder
</commit_message>
<xml_diff>
--- a/data/input/Excel_files/Soorten_bwk_afstanden.xlsx
+++ b/data/input/Excel_files/Soorten_bwk_afstanden.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1614" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1617" uniqueCount="313">
   <si>
     <t>Soort</t>
   </si>
@@ -963,6 +963,9 @@
   </si>
   <si>
     <t>Turnhouts_Vennegebied</t>
+  </si>
+  <si>
+    <t>geleluzernevlinder</t>
   </si>
 </sst>
 </file>
@@ -1281,7 +1284,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L322"/>
+  <dimension ref="A1:L323"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.109375" bestFit="1" customWidth="1"/>
@@ -10183,6 +10186,20 @@
         <v>0</v>
       </c>
     </row>
+    <row r="323" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A323" t="s">
+        <v>16</v>
+      </c>
+      <c r="B323" t="s">
+        <v>312</v>
+      </c>
+      <c r="C323" t="s">
+        <v>264</v>
+      </c>
+      <c r="D323">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I322">
     <sortState ref="A26:I100">

</xml_diff>

<commit_message>
Add Wulp, zompsprinkhaan en zadelsprinkhaan
</commit_message>
<xml_diff>
--- a/data/input/Excel_files/Soorten_bwk_afstanden.xlsx
+++ b/data/input/Excel_files/Soorten_bwk_afstanden.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1675" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1677" uniqueCount="343">
   <si>
     <t>Soort</t>
   </si>
@@ -1385,7 +1385,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:L352"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1433,7 +1432,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -1459,7 +1458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -1488,7 +1487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -1514,7 +1513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -1569,7 +1568,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -1627,7 +1626,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -1656,7 +1655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -1685,7 +1684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1743,7 +1742,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>190</v>
       </c>
@@ -1798,7 +1797,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>190</v>
       </c>
@@ -1824,7 +1823,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>190</v>
       </c>
@@ -1850,7 +1849,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>44</v>
       </c>
@@ -1879,7 +1878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>223</v>
       </c>
@@ -1937,7 +1936,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>16</v>
       </c>
@@ -1966,7 +1965,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>16</v>
       </c>
@@ -1995,7 +1994,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>44</v>
       </c>
@@ -2024,7 +2023,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>18</v>
       </c>
@@ -2050,7 +2049,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>190</v>
       </c>
@@ -2076,7 +2075,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>191</v>
       </c>
@@ -2105,7 +2104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>190</v>
       </c>
@@ -2134,7 +2133,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>190</v>
       </c>
@@ -2163,7 +2162,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>25</v>
       </c>
@@ -2192,7 +2191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>25</v>
       </c>
@@ -2221,7 +2220,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>25</v>
       </c>
@@ -2279,7 +2278,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>16</v>
       </c>
@@ -2308,7 +2307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>16</v>
       </c>
@@ -2337,7 +2336,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>16</v>
       </c>
@@ -2366,7 +2365,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>190</v>
       </c>
@@ -2392,7 +2391,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>190</v>
       </c>
@@ -2418,7 +2417,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>25</v>
       </c>
@@ -2447,7 +2446,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>25</v>
       </c>
@@ -2476,7 +2475,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>25</v>
       </c>
@@ -2534,7 +2533,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>16</v>
       </c>
@@ -2560,7 +2559,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>191</v>
       </c>
@@ -2586,7 +2585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>191</v>
       </c>
@@ -2615,7 +2614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>191</v>
       </c>
@@ -2644,7 +2643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>44</v>
       </c>
@@ -2702,7 +2701,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>44</v>
       </c>
@@ -2731,7 +2730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>44</v>
       </c>
@@ -2818,7 +2817,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>44</v>
       </c>
@@ -2847,7 +2846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>190</v>
       </c>
@@ -2873,7 +2872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>44</v>
       </c>
@@ -2902,7 +2901,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>16</v>
       </c>
@@ -2931,7 +2930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>191</v>
       </c>
@@ -2960,7 +2959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>190</v>
       </c>
@@ -2986,7 +2985,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>190</v>
       </c>
@@ -3041,7 +3040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>44</v>
       </c>
@@ -3070,7 +3069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>191</v>
       </c>
@@ -3099,7 +3098,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>191</v>
       </c>
@@ -3125,7 +3124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>191</v>
       </c>
@@ -3151,7 +3150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>191</v>
       </c>
@@ -3177,7 +3176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>191</v>
       </c>
@@ -3203,7 +3202,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>191</v>
       </c>
@@ -3229,7 +3228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>44</v>
       </c>
@@ -3258,7 +3257,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>190</v>
       </c>
@@ -3284,7 +3283,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="68" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>25</v>
       </c>
@@ -3310,7 +3309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>25</v>
       </c>
@@ -3339,7 +3338,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>25</v>
       </c>
@@ -3368,7 +3367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>190</v>
       </c>
@@ -3397,7 +3396,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>190</v>
       </c>
@@ -3423,7 +3422,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>32</v>
       </c>
@@ -3452,7 +3451,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>190</v>
       </c>
@@ -3481,7 +3480,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>16</v>
       </c>
@@ -3494,8 +3493,23 @@
       <c r="D75">
         <v>1</v>
       </c>
-    </row>
-    <row r="76" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+      <c r="E75">
+        <v>50</v>
+      </c>
+      <c r="F75">
+        <v>5000</v>
+      </c>
+      <c r="G75" t="s">
+        <v>310</v>
+      </c>
+      <c r="H75" t="s">
+        <v>291</v>
+      </c>
+      <c r="I75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>16</v>
       </c>
@@ -3524,7 +3538,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>190</v>
       </c>
@@ -3550,7 +3564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>40</v>
       </c>
@@ -3579,7 +3593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>44</v>
       </c>
@@ -3608,7 +3622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>25</v>
       </c>
@@ -3637,7 +3651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>25</v>
       </c>
@@ -3663,7 +3677,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>25</v>
       </c>
@@ -3689,7 +3703,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>25</v>
       </c>
@@ -3715,7 +3729,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>25</v>
       </c>
@@ -3744,7 +3758,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>25</v>
       </c>
@@ -3770,7 +3784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>44</v>
       </c>
@@ -3799,7 +3813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>18</v>
       </c>
@@ -3854,7 +3868,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>25</v>
       </c>
@@ -3883,7 +3897,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>25</v>
       </c>
@@ -3909,7 +3923,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>21</v>
       </c>
@@ -3938,7 +3952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>21</v>
       </c>
@@ -3967,7 +3981,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>190</v>
       </c>
@@ -3993,7 +4007,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>190</v>
       </c>
@@ -4022,7 +4036,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>190</v>
       </c>
@@ -4049,7 +4063,7 @@
       </c>
       <c r="L95" s="1"/>
     </row>
-    <row r="96" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>190</v>
       </c>
@@ -4075,7 +4089,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>190</v>
       </c>
@@ -4101,7 +4115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>190</v>
       </c>
@@ -4130,7 +4144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>190</v>
       </c>
@@ -4156,7 +4170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>190</v>
       </c>
@@ -4182,7 +4196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>190</v>
       </c>
@@ -4237,7 +4251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>16</v>
       </c>
@@ -4266,7 +4280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>41</v>
       </c>
@@ -4353,7 +4367,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>190</v>
       </c>
@@ -4379,7 +4393,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>190</v>
       </c>
@@ -4405,7 +4419,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>16</v>
       </c>
@@ -4463,7 +4477,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>190</v>
       </c>
@@ -4489,7 +4503,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>190</v>
       </c>
@@ -4518,7 +4532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>190</v>
       </c>
@@ -4547,7 +4561,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>42</v>
       </c>
@@ -4573,7 +4587,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>44</v>
       </c>
@@ -4602,7 +4616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>190</v>
       </c>
@@ -4628,7 +4642,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>190</v>
       </c>
@@ -4654,7 +4668,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>191</v>
       </c>
@@ -4680,7 +4694,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>191</v>
       </c>
@@ -4706,7 +4720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>18</v>
       </c>
@@ -4732,7 +4746,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>16</v>
       </c>
@@ -4790,7 +4804,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>18</v>
       </c>
@@ -4816,7 +4830,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>16</v>
       </c>
@@ -4845,7 +4859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>16</v>
       </c>
@@ -4874,7 +4888,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>16</v>
       </c>
@@ -4932,7 +4946,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>44</v>
       </c>
@@ -4961,7 +4975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>25</v>
       </c>
@@ -4990,7 +5004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>25</v>
       </c>
@@ -5019,7 +5033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>25</v>
       </c>
@@ -5048,7 +5062,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>190</v>
       </c>
@@ -5074,7 +5088,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>16</v>
       </c>
@@ -5100,7 +5114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>190</v>
       </c>
@@ -5126,7 +5140,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>18</v>
       </c>
@@ -5152,7 +5166,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>18</v>
       </c>
@@ -5178,7 +5192,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>16</v>
       </c>
@@ -5207,7 +5221,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>25</v>
       </c>
@@ -5236,7 +5250,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>25</v>
       </c>
@@ -5262,7 +5276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>190</v>
       </c>
@@ -5317,7 +5331,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>16</v>
       </c>
@@ -5375,7 +5389,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>16</v>
       </c>
@@ -5404,7 +5418,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>16</v>
       </c>
@@ -5462,7 +5476,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>190</v>
       </c>
@@ -5517,7 +5531,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="149" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>44</v>
       </c>
@@ -5546,7 +5560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>190</v>
       </c>
@@ -5572,7 +5586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>190</v>
       </c>
@@ -5598,7 +5612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>190</v>
       </c>
@@ -5653,7 +5667,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>44</v>
       </c>
@@ -5711,7 +5725,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>190</v>
       </c>
@@ -5737,7 +5751,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>190</v>
       </c>
@@ -5763,7 +5777,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>18</v>
       </c>
@@ -5789,7 +5803,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>18</v>
       </c>
@@ -5844,7 +5858,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>190</v>
       </c>
@@ -5870,7 +5884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>16</v>
       </c>
@@ -5899,7 +5913,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>16</v>
       </c>
@@ -5928,7 +5942,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="164" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>44</v>
       </c>
@@ -5957,7 +5971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>190</v>
       </c>
@@ -5983,7 +5997,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="166" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>190</v>
       </c>
@@ -6038,7 +6052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>190</v>
       </c>
@@ -6093,7 +6107,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>44</v>
       </c>
@@ -6122,7 +6136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>190</v>
       </c>
@@ -6148,7 +6162,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>190</v>
       </c>
@@ -6177,7 +6191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>190</v>
       </c>
@@ -6203,7 +6217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>190</v>
       </c>
@@ -6229,7 +6243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>190</v>
       </c>
@@ -6255,7 +6269,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="176" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>44</v>
       </c>
@@ -6284,7 +6298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>44</v>
       </c>
@@ -6342,7 +6356,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="179" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>40</v>
       </c>
@@ -6371,7 +6385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>190</v>
       </c>
@@ -6397,7 +6411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>190</v>
       </c>
@@ -6423,7 +6437,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>18</v>
       </c>
@@ -6449,7 +6463,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="183" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>44</v>
       </c>
@@ -6536,7 +6550,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="186" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>25</v>
       </c>
@@ -6565,7 +6579,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="187" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>25</v>
       </c>
@@ -6594,7 +6608,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>25</v>
       </c>
@@ -6623,7 +6637,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="189" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>44</v>
       </c>
@@ -6652,7 +6666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>190</v>
       </c>
@@ -6678,7 +6692,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="191" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>190</v>
       </c>
@@ -6704,7 +6718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>16</v>
       </c>
@@ -6759,7 +6773,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="194" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>223</v>
       </c>
@@ -6788,7 +6802,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="195" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>190</v>
       </c>
@@ -6817,7 +6831,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="196" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>190</v>
       </c>
@@ -6843,7 +6857,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="197" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>190</v>
       </c>
@@ -6869,7 +6883,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="198" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>43</v>
       </c>
@@ -6895,7 +6909,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>43</v>
       </c>
@@ -6921,7 +6935,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>25</v>
       </c>
@@ -6947,7 +6961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>25</v>
       </c>
@@ -6973,7 +6987,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>25</v>
       </c>
@@ -6999,7 +7013,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>25</v>
       </c>
@@ -7028,7 +7042,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="204" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>25</v>
       </c>
@@ -7057,7 +7071,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>25</v>
       </c>
@@ -7115,7 +7129,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="207" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>190</v>
       </c>
@@ -7141,7 +7155,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>190</v>
       </c>
@@ -7167,7 +7181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>44</v>
       </c>
@@ -7196,7 +7210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>190</v>
       </c>
@@ -7251,7 +7265,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="212" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>44</v>
       </c>
@@ -7280,7 +7294,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>43</v>
       </c>
@@ -7306,7 +7320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>18</v>
       </c>
@@ -7332,7 +7346,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="215" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>18</v>
       </c>
@@ -7358,7 +7372,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="216" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>44</v>
       </c>
@@ -7387,7 +7401,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>190</v>
       </c>
@@ -7413,7 +7427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="218" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>44</v>
       </c>
@@ -7442,7 +7456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>190</v>
       </c>
@@ -7468,7 +7482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>190</v>
       </c>
@@ -7495,7 +7509,7 @@
       </c>
       <c r="L220" s="1"/>
     </row>
-    <row r="221" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>16</v>
       </c>
@@ -7521,7 +7535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>190</v>
       </c>
@@ -7547,7 +7561,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>190</v>
       </c>
@@ -7573,7 +7587,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="224" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>190</v>
       </c>
@@ -7599,7 +7613,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="225" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>190</v>
       </c>
@@ -7625,7 +7639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>25</v>
       </c>
@@ -7651,7 +7665,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>25</v>
       </c>
@@ -7706,7 +7720,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="229" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>190</v>
       </c>
@@ -7732,7 +7746,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="230" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>190</v>
       </c>
@@ -7758,7 +7772,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="231" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>21</v>
       </c>
@@ -7836,7 +7850,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="234" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>190</v>
       </c>
@@ -7862,7 +7876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="235" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>190</v>
       </c>
@@ -7888,7 +7902,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="236" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>18</v>
       </c>
@@ -7911,7 +7925,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="237" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>18</v>
       </c>
@@ -7937,7 +7951,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="238" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>223</v>
       </c>
@@ -7966,7 +7980,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="239" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>44</v>
       </c>
@@ -8024,7 +8038,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="241" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>25</v>
       </c>
@@ -8108,7 +8122,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="244" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>190</v>
       </c>
@@ -8134,7 +8148,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="245" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>190</v>
       </c>
@@ -8160,7 +8174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="246" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>223</v>
       </c>
@@ -8189,7 +8203,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="247" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>16</v>
       </c>
@@ -8215,7 +8229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="248" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>25</v>
       </c>
@@ -8244,7 +8258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="249" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>25</v>
       </c>
@@ -8273,7 +8287,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="250" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>25</v>
       </c>
@@ -8302,7 +8316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="251" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>190</v>
       </c>
@@ -8328,7 +8342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="252" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>190</v>
       </c>
@@ -8357,7 +8371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="253" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>44</v>
       </c>
@@ -8386,7 +8400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="254" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>190</v>
       </c>
@@ -8412,7 +8426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="255" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>190</v>
       </c>
@@ -8438,7 +8452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="256" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>190</v>
       </c>
@@ -8464,7 +8478,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>190</v>
       </c>
@@ -8490,7 +8504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="258" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
         <v>190</v>
       </c>
@@ -8516,7 +8530,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="259" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>190</v>
       </c>
@@ -8542,7 +8556,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="260" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>190</v>
       </c>
@@ -8571,7 +8585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="261" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>16</v>
       </c>
@@ -8597,7 +8611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="262" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>190</v>
       </c>
@@ -8623,7 +8637,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="263" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>190</v>
       </c>
@@ -8678,7 +8692,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="265" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>25</v>
       </c>
@@ -8704,7 +8718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="266" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>25</v>
       </c>
@@ -8759,7 +8773,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="268" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>16</v>
       </c>
@@ -8843,7 +8857,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="271" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>223</v>
       </c>
@@ -8872,7 +8886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="272" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
         <v>16</v>
       </c>
@@ -8901,7 +8915,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="273" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>191</v>
       </c>
@@ -8927,7 +8941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="274" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>190</v>
       </c>
@@ -8953,7 +8967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="275" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>25</v>
       </c>
@@ -8982,7 +8996,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="276" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
         <v>25</v>
       </c>
@@ -9011,7 +9025,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="277" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="277" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
         <v>25</v>
       </c>
@@ -9040,7 +9054,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="278" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
         <v>25</v>
       </c>
@@ -9069,7 +9083,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="279" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>21</v>
       </c>
@@ -9095,7 +9109,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="280" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>190</v>
       </c>
@@ -9121,7 +9135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="281" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>190</v>
       </c>
@@ -9147,7 +9161,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="282" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="282" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>21</v>
       </c>
@@ -9173,7 +9187,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="283" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>21</v>
       </c>
@@ -9228,7 +9242,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="285" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>18</v>
       </c>
@@ -9254,7 +9268,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="286" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>25</v>
       </c>
@@ -9283,7 +9297,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="287" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>25</v>
       </c>
@@ -9312,7 +9326,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="288" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>25</v>
       </c>
@@ -9341,7 +9355,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="289" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>18</v>
       </c>
@@ -9370,7 +9384,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="290" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
         <v>44</v>
       </c>
@@ -9457,7 +9471,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="293" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="293" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
         <v>190</v>
       </c>
@@ -9512,7 +9526,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="295" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
         <v>190</v>
       </c>
@@ -9538,7 +9552,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="296" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>191</v>
       </c>
@@ -9567,7 +9581,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="297" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="297" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
         <v>44</v>
       </c>
@@ -9596,7 +9610,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="298" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="298" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>44</v>
       </c>
@@ -9625,7 +9639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="299" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>223</v>
       </c>
@@ -9683,7 +9697,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="301" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>190</v>
       </c>
@@ -9709,7 +9723,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="302" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>190</v>
       </c>
@@ -9735,7 +9749,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="303" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>190</v>
       </c>
@@ -9761,7 +9775,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="304" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>190</v>
       </c>
@@ -9816,7 +9830,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="306" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>190</v>
       </c>
@@ -9900,7 +9914,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="309" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
         <v>44</v>
       </c>
@@ -9929,7 +9943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="310" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
         <v>190</v>
       </c>
@@ -9955,7 +9969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="311" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
         <v>190</v>
       </c>
@@ -9981,7 +9995,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="312" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
         <v>190</v>
       </c>
@@ -10007,7 +10021,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="313" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
         <v>223</v>
       </c>
@@ -10036,7 +10050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="314" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="314" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
         <v>44</v>
       </c>
@@ -10065,7 +10079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="315" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
         <v>43</v>
       </c>
@@ -10091,7 +10105,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="316" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
         <v>16</v>
       </c>
@@ -10117,7 +10131,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="317" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
         <v>223</v>
       </c>
@@ -10146,7 +10160,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="318" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
         <v>190</v>
       </c>
@@ -10172,7 +10186,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="319" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A319" t="s">
         <v>190</v>
       </c>
@@ -10198,7 +10212,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="320" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A320" t="s">
         <v>190</v>
       </c>
@@ -10224,7 +10238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="321" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A321" t="s">
         <v>190</v>
       </c>
@@ -10250,7 +10264,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="322" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A322" t="s">
         <v>190</v>
       </c>
@@ -10276,7 +10290,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="323" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A323" t="s">
         <v>223</v>
       </c>
@@ -10305,7 +10319,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="324" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A324" t="s">
         <v>342</v>
       </c>
@@ -10313,7 +10327,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="325" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="325" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A325" t="s">
         <v>41</v>
       </c>
@@ -10321,7 +10335,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="326" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A326" t="s">
         <v>190</v>
       </c>
@@ -10329,7 +10343,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="327" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A327" t="s">
         <v>342</v>
       </c>
@@ -10337,7 +10351,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="328" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A328" t="s">
         <v>342</v>
       </c>
@@ -10345,7 +10359,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="329" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A329" t="s">
         <v>44</v>
       </c>
@@ -10362,7 +10376,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="330" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A330" t="s">
         <v>342</v>
       </c>
@@ -10370,7 +10384,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="331" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A331" t="s">
         <v>44</v>
       </c>
@@ -10387,7 +10401,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="332" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="332" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A332" t="s">
         <v>342</v>
       </c>
@@ -10395,7 +10409,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="333" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A333" t="s">
         <v>342</v>
       </c>
@@ -10403,7 +10417,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="334" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A334" t="s">
         <v>342</v>
       </c>
@@ -10411,7 +10425,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="335" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A335" t="s">
         <v>342</v>
       </c>
@@ -10419,7 +10433,7 @@
         <v>324</v>
       </c>
     </row>
-    <row r="336" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="336" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A336" t="s">
         <v>44</v>
       </c>
@@ -10436,7 +10450,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="337" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="337" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A337" t="s">
         <v>342</v>
       </c>
@@ -10444,7 +10458,7 @@
         <v>326</v>
       </c>
     </row>
-    <row r="338" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="338" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A338" t="s">
         <v>44</v>
       </c>
@@ -10461,7 +10475,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="339" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A339" t="s">
         <v>44</v>
       </c>
@@ -10478,7 +10492,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="340" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="340" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A340" t="s">
         <v>342</v>
       </c>
@@ -10486,7 +10500,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="341" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="341" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A341" t="s">
         <v>41</v>
       </c>
@@ -10494,7 +10508,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="342" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="342" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A342" t="s">
         <v>342</v>
       </c>
@@ -10502,7 +10516,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="343" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="343" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A343" t="s">
         <v>342</v>
       </c>
@@ -10510,7 +10524,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="344" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A344" t="s">
         <v>41</v>
       </c>
@@ -10518,7 +10532,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="345" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="345" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A345" t="s">
         <v>342</v>
       </c>
@@ -10526,7 +10540,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="346" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A346" t="s">
         <v>342</v>
       </c>
@@ -10534,7 +10548,7 @@
         <v>335</v>
       </c>
     </row>
-    <row r="347" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A347" t="s">
         <v>41</v>
       </c>
@@ -10542,7 +10556,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="348" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A348" t="s">
         <v>44</v>
       </c>
@@ -10559,7 +10573,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="349" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="349" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A349" t="s">
         <v>342</v>
       </c>
@@ -10567,7 +10581,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="350" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A350" t="s">
         <v>342</v>
       </c>
@@ -10575,7 +10589,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="351" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A351" t="s">
         <v>190</v>
       </c>
@@ -10583,7 +10597,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="352" spans="1:6" hidden="1" x14ac:dyDescent="0.3">
+    <row r="352" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A352" t="s">
         <v>25</v>
       </c>
@@ -10593,16 +10607,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:I352">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Planten"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="8">
-      <filters>
-        <filter val="1"/>
-      </filters>
-    </filterColumn>
     <sortState ref="A2:I323">
       <sortCondition ref="B1:B323"/>
     </sortState>

</xml_diff>

<commit_message>
Update locations waarnemingen and add shapefiles
</commit_message>
<xml_diff>
--- a/data/input/Excel_files/Soorten_bwk_afstanden.xlsx
+++ b/data/input/Excel_files/Soorten_bwk_afstanden.xlsx
@@ -1463,7 +1463,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -1544,7 +1544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>44</v>
       </c>
@@ -1602,7 +1602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>44</v>
       </c>
@@ -1631,7 +1631,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>341</v>
       </c>
@@ -1642,7 +1642,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>41</v>
       </c>
@@ -1653,7 +1653,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1682,7 +1682,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -1711,7 +1711,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -1740,7 +1740,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>44</v>
       </c>
@@ -1769,7 +1769,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>190</v>
       </c>
@@ -1795,7 +1795,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>44</v>
       </c>
@@ -1824,7 +1824,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>190</v>
       </c>
@@ -1850,7 +1850,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>190</v>
       </c>
@@ -1876,7 +1876,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>190</v>
       </c>
@@ -1945,7 +1945,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>44</v>
       </c>
@@ -1974,7 +1974,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>16</v>
       </c>
@@ -2003,7 +2003,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>16</v>
       </c>
@@ -2087,7 +2087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>190</v>
       </c>
@@ -2113,7 +2113,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>191</v>
       </c>
@@ -2142,7 +2142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>190</v>
       </c>
@@ -2171,7 +2171,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>190</v>
       </c>
@@ -2298,7 +2298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>341</v>
       </c>
@@ -2309,7 +2309,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>44</v>
       </c>
@@ -2338,7 +2338,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>16</v>
       </c>
@@ -2367,7 +2367,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>16</v>
       </c>
@@ -2396,7 +2396,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>16</v>
       </c>
@@ -2425,7 +2425,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>190</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>190</v>
       </c>
@@ -2564,7 +2564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>44</v>
       </c>
@@ -2619,7 +2619,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>191</v>
       </c>
@@ -2645,7 +2645,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>191</v>
       </c>
@@ -2674,7 +2674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>191</v>
       </c>
@@ -2703,7 +2703,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>44</v>
       </c>
@@ -2732,7 +2732,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>44</v>
       </c>
@@ -2819,7 +2819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>44</v>
       </c>
@@ -2848,7 +2848,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>44</v>
       </c>
@@ -2961,7 +2961,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>16</v>
       </c>
@@ -2990,7 +2990,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>191</v>
       </c>
@@ -3071,7 +3071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>44</v>
       </c>
@@ -3129,7 +3129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>44</v>
       </c>
@@ -3178,7 +3178,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>191</v>
       </c>
@@ -3204,7 +3204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>191</v>
       </c>
@@ -3230,7 +3230,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>191</v>
       </c>
@@ -3256,7 +3256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>191</v>
       </c>
@@ -3272,6 +3272,9 @@
       <c r="E70">
         <v>100</v>
       </c>
+      <c r="F70">
+        <v>100000</v>
+      </c>
       <c r="G70" t="s">
         <v>273</v>
       </c>
@@ -3282,7 +3285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>191</v>
       </c>
@@ -3297,6 +3300,9 @@
       </c>
       <c r="E71">
         <v>100</v>
+      </c>
+      <c r="F71">
+        <v>100000</v>
       </c>
       <c r="G71" t="s">
         <v>273</v>
@@ -3337,7 +3343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>190</v>
       </c>
@@ -3363,7 +3369,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>341</v>
       </c>
@@ -3571,7 +3577,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>44</v>
       </c>
@@ -3591,7 +3597,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>16</v>
       </c>
@@ -3620,7 +3626,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>16</v>
       </c>
@@ -3788,7 +3794,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>25</v>
       </c>
@@ -3814,7 +3820,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>25</v>
       </c>
@@ -3840,7 +3846,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>341</v>
       </c>
@@ -3851,7 +3857,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>341</v>
       </c>
@@ -3973,7 +3979,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>44</v>
       </c>
@@ -4355,7 +4361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>341</v>
       </c>
@@ -4366,7 +4372,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>44</v>
       </c>
@@ -4395,7 +4401,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>16</v>
       </c>
@@ -4435,7 +4441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>41</v>
       </c>
@@ -4464,7 +4470,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>44</v>
       </c>
@@ -4493,7 +4499,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>44</v>
       </c>
@@ -4603,7 +4609,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>44</v>
       </c>
@@ -4632,7 +4638,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>190</v>
       </c>
@@ -4658,7 +4664,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>190</v>
       </c>
@@ -4687,7 +4693,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>190</v>
       </c>
@@ -4716,7 +4722,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>44</v>
       </c>
@@ -4880,7 +4886,7 @@
         <v>270</v>
       </c>
       <c r="D132">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="E132">
         <v>100</v>
@@ -4921,7 +4927,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>16</v>
       </c>
@@ -4950,7 +4956,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>44</v>
       </c>
@@ -5005,7 +5011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>16</v>
       </c>
@@ -5034,7 +5040,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>16</v>
       </c>
@@ -5063,7 +5069,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>16</v>
       </c>
@@ -5092,7 +5098,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>44</v>
       </c>
@@ -5150,7 +5156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>25</v>
       </c>
@@ -5179,7 +5185,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>25</v>
       </c>
@@ -5208,7 +5214,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>25</v>
       </c>
@@ -5289,7 +5295,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>190</v>
       </c>
@@ -5378,7 +5384,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>44</v>
       </c>
@@ -5482,7 +5488,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>190</v>
       </c>
@@ -5508,7 +5514,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>44</v>
       </c>
@@ -5537,7 +5543,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>16</v>
       </c>
@@ -5566,7 +5572,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>44</v>
       </c>
@@ -5586,7 +5592,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>44</v>
       </c>
@@ -5615,7 +5621,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>341</v>
       </c>
@@ -5626,7 +5632,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>41</v>
       </c>
@@ -5695,7 +5701,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>44</v>
       </c>
@@ -5750,7 +5756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>44</v>
       </c>
@@ -5779,7 +5785,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>44</v>
       </c>
@@ -5886,7 +5892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>44</v>
       </c>
@@ -5944,7 +5950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>44</v>
       </c>
@@ -6077,7 +6083,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>44</v>
       </c>
@@ -6132,7 +6138,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>16</v>
       </c>
@@ -6161,7 +6167,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="181" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>16</v>
       </c>
@@ -6219,7 +6225,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>190</v>
       </c>
@@ -6271,7 +6277,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>44</v>
       </c>
@@ -6300,7 +6306,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="186" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>190</v>
       </c>
@@ -6326,7 +6332,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="187" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>44</v>
       </c>
@@ -6384,7 +6390,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>190</v>
       </c>
@@ -6491,7 +6497,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>190</v>
       </c>
@@ -6546,7 +6552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>341</v>
       </c>
@@ -6586,7 +6592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>44</v>
       </c>
@@ -6751,7 +6757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>44</v>
       </c>
@@ -6780,7 +6786,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="204" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>44</v>
       </c>
@@ -6809,7 +6815,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>25</v>
       </c>
@@ -6838,7 +6844,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="206" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>25</v>
       </c>
@@ -6867,7 +6873,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="207" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>25</v>
       </c>
@@ -6925,7 +6931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>190</v>
       </c>
@@ -6951,7 +6957,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="210" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>341</v>
       </c>
@@ -6962,7 +6968,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="211" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>190</v>
       </c>
@@ -7014,7 +7020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>44</v>
       </c>
@@ -7072,7 +7078,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>190</v>
       </c>
@@ -7101,7 +7107,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="216" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>190</v>
       </c>
@@ -7127,7 +7133,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="217" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>190</v>
       </c>
@@ -7284,7 +7290,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>25</v>
       </c>
@@ -7313,7 +7319,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="224" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:12" hidden="1" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>25</v>
       </c>
@@ -7342,7 +7348,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="225" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>25</v>
       </c>
@@ -7371,7 +7377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="226" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>44</v>
       </c>
@@ -7426,7 +7432,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>190</v>
       </c>
@@ -7481,7 +7487,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>190</v>
       </c>
@@ -7507,7 +7513,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="231" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>44</v>
       </c>
@@ -7672,7 +7678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="237" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>190</v>
       </c>
@@ -7831,7 +7837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="243" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>190</v>
       </c>
@@ -7857,7 +7863,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="244" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>190</v>
       </c>
@@ -7972,7 +7978,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="249" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>44</v>
       </c>
@@ -8001,7 +8007,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="250" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>190</v>
       </c>
@@ -8027,7 +8033,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="251" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>190</v>
       </c>
@@ -8102,7 +8108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="254" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>44</v>
       </c>
@@ -8183,7 +8189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="257" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>341</v>
       </c>
@@ -8243,7 +8249,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="260" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>341</v>
       </c>
@@ -8341,7 +8347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="264" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>41</v>
       </c>
@@ -8352,7 +8358,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="265" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>25</v>
       </c>
@@ -8378,7 +8384,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="266" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>44</v>
       </c>
@@ -8407,7 +8413,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="267" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>44</v>
       </c>
@@ -8436,7 +8442,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="268" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>190</v>
       </c>
@@ -8462,7 +8468,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="269" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>190</v>
       </c>
@@ -8517,7 +8523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="271" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>44</v>
       </c>
@@ -8563,7 +8569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="273" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>25</v>
       </c>
@@ -8592,7 +8598,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="274" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>25</v>
       </c>
@@ -8621,7 +8627,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="275" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>25</v>
       </c>
@@ -8838,7 +8844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="283" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>190</v>
       </c>
@@ -8864,7 +8870,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="284" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
         <v>190</v>
       </c>
@@ -8890,7 +8896,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="285" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="285" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>190</v>
       </c>
@@ -8997,7 +9003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="289" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="289" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>44</v>
       </c>
@@ -9144,7 +9150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="295" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
         <v>44</v>
       </c>
@@ -9173,7 +9179,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="296" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>44</v>
       </c>
@@ -9260,7 +9266,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="299" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+    <row r="299" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>191</v>
       </c>
@@ -9312,7 +9318,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="301" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>25</v>
       </c>
@@ -9341,7 +9347,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="302" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="302" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>25</v>
       </c>
@@ -9370,7 +9376,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="303" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="303" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>25</v>
       </c>
@@ -9399,7 +9405,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="304" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="304" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>25</v>
       </c>
@@ -9558,7 +9564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="310" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
         <v>44</v>
       </c>
@@ -9758,7 +9764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="317" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
         <v>44</v>
       </c>
@@ -9787,7 +9793,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="318" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
         <v>44</v>
       </c>
@@ -9842,7 +9848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="320" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A320" t="s">
         <v>44</v>
       </c>
@@ -9871,7 +9877,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="321" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A321" t="s">
         <v>190</v>
       </c>
@@ -9926,7 +9932,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="323" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A323" t="s">
         <v>341</v>
       </c>
@@ -10024,7 +10030,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="327" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A327" t="s">
         <v>44</v>
       </c>
@@ -10053,7 +10059,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="328" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A328" t="s">
         <v>190</v>
       </c>
@@ -10079,7 +10085,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="329" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A329" t="s">
         <v>190</v>
       </c>
@@ -10105,7 +10111,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="330" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A330" t="s">
         <v>190</v>
       </c>
@@ -10131,7 +10137,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="331" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A331" t="s">
         <v>190</v>
       </c>
@@ -10186,7 +10192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="333" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="333" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A333" t="s">
         <v>190</v>
       </c>
@@ -10212,7 +10218,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="334" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A334" t="s">
         <v>44</v>
       </c>
@@ -10241,7 +10247,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="335" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A335" t="s">
         <v>44</v>
       </c>
@@ -10351,7 +10357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="339" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A339" t="s">
         <v>190</v>
       </c>
@@ -10487,7 +10493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="344" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="344" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A344" t="s">
         <v>190</v>
       </c>
@@ -10527,7 +10533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="346" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="346" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A346" t="s">
         <v>25</v>
       </c>
@@ -10538,7 +10544,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="347" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="347" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A347" t="s">
         <v>190</v>
       </c>
@@ -10564,7 +10570,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="348" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="348" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A348" t="s">
         <v>190</v>
       </c>
@@ -10616,7 +10622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="350" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="350" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A350" t="s">
         <v>190</v>
       </c>
@@ -10642,7 +10648,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="351" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="351" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
       <c r="A351" t="s">
         <v>190</v>
       </c>
@@ -10699,9 +10705,9 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:I352">
-    <filterColumn colId="8">
+    <filterColumn colId="0">
       <filters>
-        <filter val="1"/>
+        <filter val="Zoogdieren"/>
       </filters>
     </filterColumn>
     <sortState ref="A2:I352">

</xml_diff>

<commit_message>
Add last modellen Maatwerkgebieden
</commit_message>
<xml_diff>
--- a/data/input/Excel_files/Soorten_bwk_afstanden.xlsx
+++ b/data/input/Excel_files/Soorten_bwk_afstanden.xlsx
@@ -4947,6 +4947,9 @@
       <c r="E133">
         <v>50</v>
       </c>
+      <c r="F133">
+        <v>2000</v>
+      </c>
       <c r="G133" t="s">
         <v>308</v>
       </c>
@@ -6107,6 +6110,9 @@
       <c r="E176">
         <v>10</v>
       </c>
+      <c r="F176">
+        <v>1000</v>
+      </c>
       <c r="G176" t="s">
         <v>272</v>
       </c>
@@ -6133,6 +6139,9 @@
       <c r="E177">
         <v>50</v>
       </c>
+      <c r="F177">
+        <v>1000</v>
+      </c>
       <c r="G177" t="s">
         <v>272</v>
       </c>
@@ -8643,6 +8652,9 @@
       <c r="E272">
         <v>50</v>
       </c>
+      <c r="F272">
+        <v>1000</v>
+      </c>
       <c r="G272" t="s">
         <v>272</v>
       </c>
@@ -9638,6 +9650,9 @@
       <c r="E309">
         <v>50</v>
       </c>
+      <c r="F309">
+        <v>1000</v>
+      </c>
       <c r="G309" t="s">
         <v>272</v>
       </c>
@@ -9663,6 +9678,9 @@
       </c>
       <c r="E310">
         <v>50</v>
+      </c>
+      <c r="F310">
+        <v>1000</v>
       </c>
       <c r="G310" t="s">
         <v>272</v>

</xml_diff>